<commit_message>
chore: keep TikTok capture outputs local
</commit_message>
<xml_diff>
--- a/inbox-pengman/output/tiktok_account_data_2026-07-20.xlsx
+++ b/inbox-pengman/output/tiktok_account_data_2026-07-20.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accounts" sheetId="1" r:id="R7a581bec9876400e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posts" sheetId="2" r:id="R6d9847dc0d8a40d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="accounts" sheetId="1" r:id="Rdae82437f46549cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posts" sheetId="2" r:id="R9a6cffc6328d4f65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -418,7 +418,7 @@
 ask me for free astrology readings</x:v>
       </x:c>
       <x:c r="I2" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -445,7 +445,7 @@
       </x:c>
       <x:c r="H3" s="14" t="str"/>
       <x:c r="I3" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -476,7 +476,7 @@
 Send me your birthday 💕</x:v>
       </x:c>
       <x:c r="I4" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -503,13 +503,13 @@
       </x:c>
       <x:c r="H5" s="14" t="str"/>
       <x:c r="I5" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82a3f54a26dd4bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b57665feba4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -606,7 +606,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L2" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="54" hidden="0" customHeight="1">
@@ -645,7 +645,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L3" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" hidden="0" customHeight="1">
@@ -684,7 +684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" hidden="0" customHeight="1">
@@ -723,7 +723,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L5" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" hidden="0" customHeight="1">
@@ -762,7 +762,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L6" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" hidden="0" customHeight="1">
@@ -801,7 +801,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L7" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" hidden="0" customHeight="1">
@@ -840,7 +840,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L8" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" hidden="0" customHeight="1">
@@ -879,7 +879,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L9" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" hidden="0" customHeight="1">
@@ -918,7 +918,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L10" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" hidden="0" customHeight="1">
@@ -942,7 +942,7 @@
         <x:v>Read the full birth chart overview: https://www.astrologywiki.com/en/wiki/erling-haaland-birth-chart</x:v>
       </x:c>
       <x:c r="G11" s="12" t="n">
-        <x:v>800</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="H11" s="12" t="n">
         <x:v>10</x:v>
@@ -957,7 +957,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L11" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" hidden="0" customHeight="1">
@@ -981,7 +981,7 @@
         <x:v>what a great win🥳  Good night everyone  Hope that I can fall asleep tonight #worldcup #spain </x:v>
       </x:c>
       <x:c r="G12" s="12" t="n">
-        <x:v>31</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="H12" s="12" t="n">
         <x:v>1</x:v>
@@ -996,7 +996,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" hidden="0" customHeight="1">
@@ -1013,19 +1013,29 @@
       <x:c r="D13" t="str">
         <x:v>photo</x:v>
       </x:c>
-      <x:c r="E13" s="13"/>
+      <x:c r="E13" s="13" t="n">
+        <x:v>46220.14494212963</x:v>
+      </x:c>
       <x:c r="F13" s="14" t="str">
         <x:v>Astrology reading Two ♋️ sun #worldcup #messi #yamal #worldcup #astrology </x:v>
       </x:c>
       <x:c r="G13" s="12" t="n">
-        <x:v>395</x:v>
-      </x:c>
-      <x:c r="H13" s="12"/>
-      <x:c r="I13" s="12"/>
-      <x:c r="J13" s="12"/>
-      <x:c r="K13" s="12"/>
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I13" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K13" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L13" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" hidden="0" customHeight="1">
@@ -1042,19 +1052,29 @@
       <x:c r="D14" t="str">
         <x:v>photo</x:v>
       </x:c>
-      <x:c r="E14" s="13"/>
+      <x:c r="E14" s="13" t="n">
+        <x:v>46217.47293981481</x:v>
+      </x:c>
       <x:c r="F14" s="14" t="str">
         <x:v>Lamont Yamal turned 19 yesterday and plays worldcup semi today - in his own Cancer season Which team do you pick? #worldcup #france #spain #astrology #birthchart </x:v>
       </x:c>
       <x:c r="G14" s="12" t="n">
         <x:v>1902</x:v>
       </x:c>
-      <x:c r="H14" s="12"/>
-      <x:c r="I14" s="12"/>
-      <x:c r="J14" s="12"/>
-      <x:c r="K14" s="12"/>
+      <x:c r="H14" s="12" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="I14" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J14" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K14" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L14" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" hidden="0" customHeight="1">
@@ -1093,7 +1113,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="L15" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" hidden="0" customHeight="1">
@@ -1132,7 +1152,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L16" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" hidden="0" customHeight="1">
@@ -1171,7 +1191,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L17" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" hidden="0" customHeight="1">
@@ -1210,7 +1230,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L18" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" hidden="0" customHeight="1">
@@ -1249,7 +1269,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L19" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" hidden="0" customHeight="1">
@@ -1288,7 +1308,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L20" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" hidden="0" customHeight="1">
@@ -1327,13 +1347,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L21" s="13" t="n">
-        <x:v>46223.27581461806</x:v>
+        <x:v>46223.28400516204</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bbb9cfa85ec4272"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c025b49b1974927"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>